<commit_message>
Update course data names
</commit_message>
<xml_diff>
--- a/course_data/e-commerce_data.xlsx
+++ b/course_data/e-commerce_data.xlsx
@@ -1102,25 +1102,33 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5738B6F9-9951-6942-AD5B-B566DD81F22B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{5738B6F9-9951-6942-AD5B-B566DD81F22B}">
   <dimension ref="A1:D51"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" ns3:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" ns3:dyDescent="0.2">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>order_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>customer_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>product_id</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ns3:dyDescent="0.2">
       <c r="A2">
         <v>1001</v>
       </c>
@@ -1134,7 +1142,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" ns3:dyDescent="0.2">
       <c r="A3">
         <v>1002</v>
       </c>
@@ -1148,7 +1156,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" ns3:dyDescent="0.2">
       <c r="A4">
         <v>1003</v>
       </c>
@@ -1162,7 +1170,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" ns3:dyDescent="0.2">
       <c r="A5">
         <v>1004</v>
       </c>
@@ -1176,7 +1184,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" ns3:dyDescent="0.2">
       <c r="A6">
         <v>1005</v>
       </c>
@@ -1190,7 +1198,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" ns3:dyDescent="0.2">
       <c r="A7">
         <v>1006</v>
       </c>
@@ -1204,7 +1212,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" ns3:dyDescent="0.2">
       <c r="A8">
         <v>1007</v>
       </c>
@@ -1218,7 +1226,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" ns3:dyDescent="0.2">
       <c r="A9">
         <v>1008</v>
       </c>
@@ -1232,7 +1240,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" ns3:dyDescent="0.2">
       <c r="A10">
         <v>1009</v>
       </c>
@@ -1246,7 +1254,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" ns3:dyDescent="0.2">
       <c r="A11">
         <v>1010</v>
       </c>
@@ -1260,7 +1268,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" ns3:dyDescent="0.2">
       <c r="A12">
         <v>1011</v>
       </c>
@@ -1274,7 +1282,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" ns3:dyDescent="0.2">
       <c r="A13">
         <v>1012</v>
       </c>
@@ -1288,7 +1296,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" ns3:dyDescent="0.2">
       <c r="A14">
         <v>1013</v>
       </c>
@@ -1302,7 +1310,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" ns3:dyDescent="0.2">
       <c r="A15">
         <v>1014</v>
       </c>
@@ -1316,7 +1324,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" ns3:dyDescent="0.2">
       <c r="A16">
         <v>1015</v>
       </c>
@@ -1330,7 +1338,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" ns3:dyDescent="0.2">
       <c r="A17">
         <v>1016</v>
       </c>
@@ -1344,7 +1352,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" ns3:dyDescent="0.2">
       <c r="A18">
         <v>1017</v>
       </c>
@@ -1358,7 +1366,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" ns3:dyDescent="0.2">
       <c r="A19">
         <v>1018</v>
       </c>
@@ -1372,7 +1380,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" ns3:dyDescent="0.2">
       <c r="A20">
         <v>1019</v>
       </c>
@@ -1386,7 +1394,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" ns3:dyDescent="0.2">
       <c r="A21">
         <v>1020</v>
       </c>
@@ -1400,7 +1408,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4" ns3:dyDescent="0.2">
       <c r="A22">
         <v>1021</v>
       </c>
@@ -1414,7 +1422,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:4" ns3:dyDescent="0.2">
       <c r="A23">
         <v>1022</v>
       </c>
@@ -1428,7 +1436,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:4" ns3:dyDescent="0.2">
       <c r="A24">
         <v>1023</v>
       </c>
@@ -1442,7 +1450,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:4" ns3:dyDescent="0.2">
       <c r="A25">
         <v>1024</v>
       </c>
@@ -1456,7 +1464,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:4" ns3:dyDescent="0.2">
       <c r="A26">
         <v>1025</v>
       </c>
@@ -1470,7 +1478,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:4" ns3:dyDescent="0.2">
       <c r="A27">
         <v>1026</v>
       </c>
@@ -1484,7 +1492,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:4" ns3:dyDescent="0.2">
       <c r="A28">
         <v>1027</v>
       </c>
@@ -1498,7 +1506,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:4" ns3:dyDescent="0.2">
       <c r="A29">
         <v>1028</v>
       </c>
@@ -1512,7 +1520,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:4" ns3:dyDescent="0.2">
       <c r="A30">
         <v>1029</v>
       </c>
@@ -1526,7 +1534,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:4" ns3:dyDescent="0.2">
       <c r="A31">
         <v>1030</v>
       </c>
@@ -1540,7 +1548,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:4" ns3:dyDescent="0.2">
       <c r="A32">
         <v>1031</v>
       </c>
@@ -1554,7 +1562,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:4" ns3:dyDescent="0.2">
       <c r="A33">
         <v>1032</v>
       </c>
@@ -1568,7 +1576,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:4" ns3:dyDescent="0.2">
       <c r="A34">
         <v>1033</v>
       </c>
@@ -1582,7 +1590,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:4" ns3:dyDescent="0.2">
       <c r="A35">
         <v>1034</v>
       </c>
@@ -1596,7 +1604,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:4" ns3:dyDescent="0.2">
       <c r="A36">
         <v>1035</v>
       </c>
@@ -1610,7 +1618,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:4" ns3:dyDescent="0.2">
       <c r="A37">
         <v>1036</v>
       </c>
@@ -1624,7 +1632,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:4" ns3:dyDescent="0.2">
       <c r="A38">
         <v>1037</v>
       </c>
@@ -1638,7 +1646,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:4" ns3:dyDescent="0.2">
       <c r="A39">
         <v>1038</v>
       </c>
@@ -1652,7 +1660,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:4" ns3:dyDescent="0.2">
       <c r="A40">
         <v>1039</v>
       </c>
@@ -1666,7 +1674,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:4" ns3:dyDescent="0.2">
       <c r="A41">
         <v>1040</v>
       </c>
@@ -1680,7 +1688,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:4" ns3:dyDescent="0.2">
       <c r="A42">
         <v>1041</v>
       </c>
@@ -1694,7 +1702,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:4" ns3:dyDescent="0.2">
       <c r="A43">
         <v>1042</v>
       </c>
@@ -1708,7 +1716,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:4" ns3:dyDescent="0.2">
       <c r="A44">
         <v>1043</v>
       </c>
@@ -1722,7 +1730,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:4" ns3:dyDescent="0.2">
       <c r="A45">
         <v>1044</v>
       </c>
@@ -1736,7 +1744,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:4" ns3:dyDescent="0.2">
       <c r="A46">
         <v>1045</v>
       </c>
@@ -1750,7 +1758,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:4" ns3:dyDescent="0.2">
       <c r="A47">
         <v>1046</v>
       </c>
@@ -1764,7 +1772,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:4" ns3:dyDescent="0.2">
       <c r="A48">
         <v>1047</v>
       </c>
@@ -1778,7 +1786,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:4" ns3:dyDescent="0.2">
       <c r="A49">
         <v>1048</v>
       </c>
@@ -1792,7 +1800,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:4" ns3:dyDescent="0.2">
       <c r="A50">
         <v>1049</v>
       </c>
@@ -1806,7 +1814,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:4" ns3:dyDescent="0.2">
       <c r="A51">
         <v>1050</v>
       </c>
@@ -1826,239 +1834,325 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C28D3822-B3FE-8F47-AF4D-A6FD015655B0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{C28D3822-B3FE-8F47-AF4D-A6FD015655B0}">
   <dimension ref="A1:C21"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" ns3:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" ns3:dyDescent="0.2">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>customer_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ns3:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Sophia Becker</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ns3:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
-        <v>26</v>
-      </c>
-      <c r="C3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Lukas Schneider</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ns3:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Emma Fischer</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ns3:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Noah Weber</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ns3:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Mia Wagner</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ns3:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" t="s">
-        <v>22</v>
-      </c>
-      <c r="C7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Leon Hoffmann</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ns3:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Hannah Meyer</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ns3:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" t="s">
-        <v>20</v>
-      </c>
-      <c r="C9" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Finn Schulz</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ns3:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Lea Koch</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ns3:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
-      <c r="B11" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Jonas Bauer</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ns3:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
-      <c r="B12" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Anna Richter</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ns3:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
-      <c r="B13" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Elias Klein</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ns3:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
-      <c r="B14" t="s">
-        <v>15</v>
-      </c>
-      <c r="C14" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Lina Wolf</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ns3:dyDescent="0.2">
       <c r="A15">
         <v>14</v>
       </c>
-      <c r="B15" t="s">
-        <v>14</v>
-      </c>
-      <c r="C15" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Paul Neumann</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ns3:dyDescent="0.2">
       <c r="A16">
         <v>15</v>
       </c>
-      <c r="B16" t="s">
-        <v>12</v>
-      </c>
-      <c r="C16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Clara Schwarz</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ns3:dyDescent="0.2">
       <c r="A17">
         <v>16</v>
       </c>
-      <c r="B17" t="s">
-        <v>10</v>
-      </c>
-      <c r="C17" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Ben Zimmermann</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ns3:dyDescent="0.2">
       <c r="A18">
         <v>17</v>
       </c>
-      <c r="B18" t="s">
-        <v>9</v>
-      </c>
-      <c r="C18" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Marie Braun</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ns3:dyDescent="0.2">
       <c r="A19">
         <v>18</v>
       </c>
-      <c r="B19" t="s">
-        <v>7</v>
-      </c>
-      <c r="C19" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Max Hartmann</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ns3:dyDescent="0.2">
       <c r="A20">
         <v>19</v>
       </c>
-      <c r="B20" t="s">
-        <v>6</v>
-      </c>
-      <c r="C20" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Laura Lange</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ns3:dyDescent="0.2">
       <c r="A21">
         <v>20</v>
       </c>
-      <c r="B21" t="s">
-        <v>5</v>
-      </c>
-      <c r="C21" t="s">
-        <v>4</v>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Tim Krause</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2067,299 +2161,387 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6785D593-1D2F-AD42-8943-B313A121C57F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{6785D593-1D2F-AD42-8943-B313A121C57F}">
   <dimension ref="A1:D21"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" ns3:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C1" t="s">
-        <v>31</v>
-      </c>
-      <c r="D1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" ns3:dyDescent="0.2">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>product_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>product_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ns3:dyDescent="0.2">
       <c r="A2">
         <v>101</v>
       </c>
-      <c r="B2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C2" t="s">
-        <v>34</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Running Shoes</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
       </c>
       <c r="D2">
         <v>137</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" ns3:dyDescent="0.2">
       <c r="A3">
         <v>102</v>
       </c>
-      <c r="B3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C3" t="s">
-        <v>36</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Ceramic Table Lamp</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
       </c>
       <c r="D3">
         <v>68</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" ns3:dyDescent="0.2">
       <c r="A4">
         <v>103</v>
       </c>
-      <c r="B4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C4" t="s">
-        <v>38</v>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Cotton T-Shirt</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Fashion</t>
+        </is>
       </c>
       <c r="D4">
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" ns3:dyDescent="0.2">
       <c r="A5">
         <v>104</v>
       </c>
-      <c r="B5" t="s">
-        <v>39</v>
-      </c>
-      <c r="C5" t="s">
-        <v>34</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Yoga Mat</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
       </c>
       <c r="D5">
         <v>65</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" ns3:dyDescent="0.2">
       <c r="A6">
         <v>105</v>
       </c>
-      <c r="B6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C6" t="s">
-        <v>36</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Kitchen Towel Set</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
       </c>
       <c r="D6">
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" ns3:dyDescent="0.2">
       <c r="A7">
         <v>106</v>
       </c>
-      <c r="B7" t="s">
-        <v>41</v>
-      </c>
-      <c r="C7" t="s">
-        <v>38</v>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Leather Jacket</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Fashion</t>
+        </is>
       </c>
       <c r="D7">
         <v>176</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" ns3:dyDescent="0.2">
       <c r="A8">
         <v>107</v>
       </c>
-      <c r="B8" t="s">
-        <v>42</v>
-      </c>
-      <c r="C8" t="s">
-        <v>34</v>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Fitness Tracker</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
       </c>
       <c r="D8">
         <v>101</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" ns3:dyDescent="0.2">
       <c r="A9">
         <v>108</v>
       </c>
-      <c r="B9" t="s">
-        <v>43</v>
-      </c>
-      <c r="C9" t="s">
-        <v>34</v>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Mountain Backpack</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
       </c>
       <c r="D9">
         <v>146</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" ns3:dyDescent="0.2">
       <c r="A10">
         <v>109</v>
       </c>
-      <c r="B10" t="s">
-        <v>44</v>
-      </c>
-      <c r="C10" t="s">
-        <v>36</v>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Bedside Organizer</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
       </c>
       <c r="D10">
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" ns3:dyDescent="0.2">
       <c r="A11">
         <v>110</v>
       </c>
-      <c r="B11" t="s">
-        <v>45</v>
-      </c>
-      <c r="C11" t="s">
-        <v>34</v>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Training Gloves</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
       </c>
       <c r="D11">
         <v>50</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" ns3:dyDescent="0.2">
       <c r="A12">
         <v>111</v>
       </c>
-      <c r="B12" t="s">
-        <v>46</v>
-      </c>
-      <c r="C12" t="s">
-        <v>36</v>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Air Purifier</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
       </c>
       <c r="D12">
         <v>154</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" ns3:dyDescent="0.2">
       <c r="A13">
         <v>112</v>
       </c>
-      <c r="B13" t="s">
-        <v>47</v>
-      </c>
-      <c r="C13" t="s">
-        <v>48</v>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Wireless Mouse</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
       </c>
       <c r="D13">
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" ns3:dyDescent="0.2">
       <c r="A14">
         <v>113</v>
       </c>
-      <c r="B14" t="s">
-        <v>49</v>
-      </c>
-      <c r="C14" t="s">
-        <v>48</v>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Bluetooth Speaker</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
       </c>
       <c r="D14">
         <v>67</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" ns3:dyDescent="0.2">
       <c r="A15">
         <v>114</v>
       </c>
-      <c r="B15" t="s">
-        <v>50</v>
-      </c>
-      <c r="C15" t="s">
-        <v>38</v>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Denim Jeans</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Fashion</t>
+        </is>
       </c>
       <c r="D15">
         <v>108</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" ns3:dyDescent="0.2">
       <c r="A16">
         <v>115</v>
       </c>
-      <c r="B16" t="s">
-        <v>51</v>
-      </c>
-      <c r="C16" t="s">
-        <v>38</v>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Knit Scarf</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Fashion</t>
+        </is>
       </c>
       <c r="D16">
         <v>45</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" ns3:dyDescent="0.2">
       <c r="A17">
         <v>116</v>
       </c>
-      <c r="B17" t="s">
-        <v>52</v>
-      </c>
-      <c r="C17" t="s">
-        <v>36</v>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Scented Candle</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
       </c>
       <c r="D17">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" ns3:dyDescent="0.2">
       <c r="A18">
         <v>117</v>
       </c>
-      <c r="B18" t="s">
-        <v>53</v>
-      </c>
-      <c r="C18" t="s">
-        <v>48</v>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Noise-Canceling Headphones</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
       </c>
       <c r="D18">
         <v>110</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" ns3:dyDescent="0.2">
       <c r="A19">
         <v>118</v>
       </c>
-      <c r="B19" t="s">
-        <v>54</v>
-      </c>
-      <c r="C19" t="s">
-        <v>38</v>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Wool Coat</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Fashion</t>
+        </is>
       </c>
       <c r="D19">
         <v>193</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" ns3:dyDescent="0.2">
       <c r="A20">
         <v>119</v>
       </c>
-      <c r="B20" t="s">
-        <v>55</v>
-      </c>
-      <c r="C20" t="s">
-        <v>38</v>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Designer Handbag</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Fashion</t>
+        </is>
       </c>
       <c r="D20">
         <v>183</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" ns3:dyDescent="0.2">
       <c r="A21">
         <v>120</v>
       </c>
-      <c r="B21" t="s">
-        <v>56</v>
-      </c>
-      <c r="C21" t="s">
-        <v>34</v>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Water Bottle</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
       </c>
       <c r="D21">
         <v>33</v>

</xml_diff>